<commit_message>
Update monthly Royal Gazette spreadsheet
</commit_message>
<xml_diff>
--- a/data/raw/monthly-latest.xlsx
+++ b/data/raw/monthly-latest.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="636">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="651">
   <si>
     <t>วันที่</t>
   </si>
@@ -1923,6 +1923,51 @@
   </si>
   <si>
     <t>https://ratchakitcha.soc.go.th/documents/132025.pdf</t>
+  </si>
+  <si>
+    <t>03/10/2026</t>
+  </si>
+  <si>
+    <t>ประกาศสำนักนายกรัฐมนตรี เรื่อง แต่งตั้งข้าราชการพลเรือนสามัญ [สำนักนายกรัฐมนตรี : นายณัฐพล รังสิตพล]</t>
+  </si>
+  <si>
+    <t>https://ratchakitcha.soc.go.th/documents/133740.pdf</t>
+  </si>
+  <si>
+    <t>กระทู้ถามของสมาชิกสภาผู้แทนราษฎร กระทู้ถามที่ 154 ร. เรื่อง มาตรการป้องกันการแพร่ระบาดของโรคไข้เลือดออก และแนวทางการจัดการวัคซีน Qdenga [ของนายเอกราช อุดมอำนวย สมาชิกสภาผู้แทนราษฎร พรรคประชาชน กรุงเทพมหานคร]</t>
+  </si>
+  <si>
+    <t>https://ratchakitcha.soc.go.th/documents/130925.pdf</t>
+  </si>
+  <si>
+    <t>กระทู้ถามของสมาชิกสภาผู้แทนราษฎร กระทู้ถามที่ 052/ร. เรื่อง แนวทางและมาตรการเยียวยาป้องกันผู้ประกอบการและชาวบ้านบริเวณโดยรอบที่ได้รับผลกระทบจากการก่อสร้างโครงการรถไฟฟ้าใต้ดินสายสีส้ม (ตะวันตก) เริ่มต้น ณ บริเวณถนนเพชรบุรี กรุงเทพมหานคร [นายเสกสิทธิ์ แย้มสงวนศักดิ์ สมาชิกสภาผู้แทนราษฎร พรรคประชาชน กรุงเทพมหานคร]</t>
+  </si>
+  <si>
+    <t>https://ratchakitcha.soc.go.th/documents/131108.pdf</t>
+  </si>
+  <si>
+    <t>กระทู้ถามของสมาชิกสภาผู้แทนราษฎร กระทู้ถามที่ 099/ร. เรื่อง ขอให้พิจารณาเร่งรัดดำเนินการบรรเทาความเดือดร้อนของประชาชนผู้ใช้รถใช้ถนนจากการดำเนินโครงการก่อสร้างถนนสาย สป. 1006 อำเภอบางบ่อ และอำเภอบางเสาธง จังหวัดสมุทรปราการ ทั้งสองช่วง [ของนายเทพฤทธิ์ ภาษี สมาชิกสภาผู้แทนราษฎร พรรคประชาชน จังหวัดสมุทรปราการ]</t>
+  </si>
+  <si>
+    <t>https://ratchakitcha.soc.go.th/documents/131291.pdf</t>
+  </si>
+  <si>
+    <t>กระทู้ถามของสมาชิกสภาผู้แทนราษฎร กระทู้ถามที่ 112/ร. เรื่อง ปัญหาการไม่ได้รับการแก้ไขจากภาครัฐกรณีไม่มีรถขนส่งสาธารณะในหลายพื้นที่ของกรุงเทพมหานคร [ของนายภูริวรรธก์ ใจสำราญ สมาชิกสภาผู้แทนราษฎร พรรคประชาชน กรุงเทพมหานคร]</t>
+  </si>
+  <si>
+    <t>https://ratchakitcha.soc.go.th/documents/131292.pdf</t>
+  </si>
+  <si>
+    <t>กระทู้ถามของสมาชิกสภาผู้แทนราษฎร กระทู้ถามที่ 113/ร. เรื่อง ขอทราบแนวทางการบริหารจัดการพื้นที่และโครงข่ายจราจรต่อเนื่องของทางหลวงพิเศษหมายเลข 81 (บางใหญ่ – กาญจนบุรี) เพื่อบรรเทาผลกระทบและพัฒนาคุณภาพชีวิตของประชาชนในพื้นที่อำเภอบางใหญ่ จังหวัดนนทบุรี [ของนายสุทัศน์ มีศิริ สมาชิกสภาผู้แทนราษฎร พรรคประชาชน จังหวัดนนทบุรี]</t>
+  </si>
+  <si>
+    <t>https://ratchakitcha.soc.go.th/documents/131293.pdf</t>
+  </si>
+  <si>
+    <t>กระทู้ถามของสมาชิกสภาผู้แทนราษฎร กระทู้ถามที่ 114/ร. เรื่อง แนวทางแก้ไขปัญหาความเดือดร้อนให้กับประชาชนที่ได้รับผลกระทบจากการดำเนินการโครงการฟลัดเวย์ (Flood way) และโครงการนำสายสื่อสารและสายไฟฟ้าลงดิน [ของนายกรณ์ มีดี สมาชิกสภาผู้แทนราษฎร พรรคประชาชน จังหวัดนนทบุรี]</t>
+  </si>
+  <si>
+    <t>https://ratchakitcha.soc.go.th/documents/131294.pdf</t>
   </si>
 </sst>
 </file>
@@ -2269,7 +2314,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:H313"/>
+  <dimension ref="A1:H320"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12.02" customWidth="true" style="0"/>
@@ -9773,12 +9818,180 @@
       </c>
     </row>
     <row r="313" spans="1:8">
-      <c r="A313" s="2"/>
-      <c r="C313" s="1"/>
-      <c r="D313" s="1"/>
-      <c r="E313" s="1"/>
-      <c r="F313" s="1"/>
+      <c r="A313" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="B313" t="s">
+        <v>637</v>
+      </c>
+      <c r="C313" s="1">
+        <v>143</v>
+      </c>
+      <c r="D313" s="1">
+        <v>240</v>
+      </c>
+      <c r="E313" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F313" s="1">
+        <v>1</v>
+      </c>
       <c r="G313" s="1"/>
+      <c r="H313" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="314" spans="1:8">
+      <c r="A314" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="B314" t="s">
+        <v>639</v>
+      </c>
+      <c r="C314" s="1">
+        <v>143</v>
+      </c>
+      <c r="D314" s="1">
+        <v>240</v>
+      </c>
+      <c r="E314" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F314" s="1">
+        <v>2</v>
+      </c>
+      <c r="G314" s="1"/>
+      <c r="H314" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="315" spans="1:8">
+      <c r="A315" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="B315" t="s">
+        <v>641</v>
+      </c>
+      <c r="C315" s="1">
+        <v>143</v>
+      </c>
+      <c r="D315" s="1">
+        <v>240</v>
+      </c>
+      <c r="E315" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F315" s="1">
+        <v>10</v>
+      </c>
+      <c r="G315" s="1"/>
+      <c r="H315" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="316" spans="1:8">
+      <c r="A316" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="B316" t="s">
+        <v>643</v>
+      </c>
+      <c r="C316" s="1">
+        <v>143</v>
+      </c>
+      <c r="D316" s="1">
+        <v>240</v>
+      </c>
+      <c r="E316" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F316" s="1">
+        <v>19</v>
+      </c>
+      <c r="G316" s="1"/>
+      <c r="H316" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="317" spans="1:8">
+      <c r="A317" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="B317" t="s">
+        <v>645</v>
+      </c>
+      <c r="C317" s="1">
+        <v>143</v>
+      </c>
+      <c r="D317" s="1">
+        <v>240</v>
+      </c>
+      <c r="E317" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F317" s="1">
+        <v>25</v>
+      </c>
+      <c r="G317" s="1"/>
+      <c r="H317" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="318" spans="1:8">
+      <c r="A318" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="B318" t="s">
+        <v>647</v>
+      </c>
+      <c r="C318" s="1">
+        <v>143</v>
+      </c>
+      <c r="D318" s="1">
+        <v>240</v>
+      </c>
+      <c r="E318" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F318" s="1">
+        <v>30</v>
+      </c>
+      <c r="G318" s="1"/>
+      <c r="H318" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="319" spans="1:8">
+      <c r="A319" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="B319" t="s">
+        <v>649</v>
+      </c>
+      <c r="C319" s="1">
+        <v>143</v>
+      </c>
+      <c r="D319" s="1">
+        <v>240</v>
+      </c>
+      <c r="E319" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F319" s="1">
+        <v>35</v>
+      </c>
+      <c r="G319" s="1"/>
+      <c r="H319" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="320" spans="1:8">
+      <c r="A320" s="2"/>
+      <c r="C320" s="1"/>
+      <c r="D320" s="1"/>
+      <c r="E320" s="1"/>
+      <c r="F320" s="1"/>
+      <c r="G320" s="1"/>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>

</xml_diff>